<commit_message>
chore(docs): update edt contents
</commit_message>
<xml_diff>
--- a/docs/edt_entrega_2.xlsx
+++ b/docs/edt_entrega_2.xlsx
@@ -992,7 +992,7 @@
       <c r="B11" s="15" t="inlineStr"/>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>⬛ Análisis de Requisitos Completado</t>
+          <t>Análisis de Requisitos Completado</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
@@ -1272,7 +1272,7 @@
       <c r="B17" s="15" t="inlineStr"/>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>⬛ Diseño Completado</t>
+          <t>Diseño Completado</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -2062,7 +2062,7 @@
       <c r="B34" s="15" t="inlineStr"/>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>⬛ Sistema Aprobado para Despliegue</t>
+          <t>Sistema Aprobado para Despliegue</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
@@ -2534,7 +2534,7 @@
       <c r="B44" s="15" t="inlineStr"/>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>⬛ Cierre Formal del Proyecto</t>
+          <t>Cierre Formal del Proyecto</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">

</xml_diff>

<commit_message>
chore(docs): align schedule, totals and presentation
</commit_message>
<xml_diff>
--- a/docs/edt_entrega_2.xlsx
+++ b/docs/edt_entrega_2.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MM-YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -121,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,7 +136,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -146,7 +145,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -155,7 +154,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -164,13 +163,25 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -561,35 +572,13 @@
           <t>Cronograma del Proyecto — Consultorio Digital</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ICI-513 Gestión de Proyectos Informáticos · Universidad de Valparaíso · Fecha base: 10-03-2026</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
+          <t>ICI-513 Gestión de Proyectos Informáticos · Universidad de Valparaíso · Fecha base: 10-03-2026 · Dedicación part-time: ~2 h/día por persona responsable</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -674,11 +663,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="19" t="n">
         <v>46091</v>
       </c>
-      <c r="F4" s="7" t="n">
-        <v>46097</v>
+      <c r="F4" s="19" t="n">
+        <v>46103</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -720,11 +709,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="20" t="n">
         <v>46091</v>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>46092</v>
+      <c r="F5" s="20" t="n">
+        <v>46094</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
@@ -766,11 +755,11 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
-        <v>46093</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>46094</v>
+      <c r="E6" s="21" t="n">
+        <v>46095</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>46098</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
@@ -812,11 +801,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n">
-        <v>46095</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>46096</v>
+      <c r="E7" s="20" t="n">
+        <v>46099</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>46103</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
@@ -862,11 +851,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
-        <v>46097</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>46103</v>
+      <c r="E8" s="19" t="n">
+        <v>46104</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>46118</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
@@ -908,11 +897,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
-        <v>46097</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>46099</v>
+      <c r="E9" s="20" t="n">
+        <v>46104</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>46110</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -954,11 +943,11 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>46100</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>46101</v>
+      <c r="E10" s="21" t="n">
+        <v>46111</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>46115</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -1000,11 +989,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E11" s="16" t="n">
-        <v>46103</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>46103</v>
+      <c r="E11" s="22" t="n">
+        <v>46118</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>46118</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1050,11 +1039,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
-        <v>46104</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>46110</v>
+      <c r="E12" s="19" t="n">
+        <v>46119</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>46121</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -1096,11 +1085,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
-        <v>46104</v>
-      </c>
-      <c r="F13" s="10" t="n">
-        <v>46105</v>
+      <c r="E13" s="20" t="n">
+        <v>46119</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>46119</v>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
@@ -1142,15 +1131,15 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E14" s="13" t="n">
-        <v>46106</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>46107</v>
+      <c r="E14" s="21" t="n">
+        <v>46119</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>46120</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="H14" s="11" t="n">
@@ -1188,11 +1177,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n">
-        <v>46108</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>46108</v>
+      <c r="E15" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>46120</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -1234,11 +1223,11 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n">
-        <v>46109</v>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>46109</v>
+      <c r="E16" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>46121</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
@@ -1280,11 +1269,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E17" s="16" t="n">
-        <v>46110</v>
-      </c>
-      <c r="F17" s="16" t="n">
-        <v>46110</v>
+      <c r="E17" s="22" t="n">
+        <v>46121</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>46121</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -1330,11 +1319,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E18" s="7" t="n">
-        <v>46111</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>46132</v>
+      <c r="E18" s="19" t="n">
+        <v>46122</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>46146</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
@@ -1376,11 +1365,11 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
-        <v>46111</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>46114</v>
+      <c r="E19" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <v>46128</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -1422,11 +1411,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E20" s="13" t="n">
-        <v>46115</v>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>46115</v>
+      <c r="E20" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>46132</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
@@ -1468,11 +1457,11 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n">
-        <v>46116</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>46116</v>
+      <c r="E21" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>46134</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -1514,11 +1503,11 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E22" s="13" t="n">
-        <v>46111</v>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>46113</v>
+      <c r="E22" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>46126</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
@@ -1560,11 +1549,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E23" s="10" t="n">
-        <v>46117</v>
-      </c>
-      <c r="F23" s="10" t="n">
-        <v>46118</v>
+      <c r="E23" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>46139</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
@@ -1606,11 +1595,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>46119</v>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>46124</v>
+      <c r="E24" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="F24" s="21" t="n">
+        <v>46143</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
@@ -1652,11 +1641,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E25" s="10" t="n">
-        <v>46125</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <v>46127</v>
+      <c r="E25" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>46145</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -1698,11 +1687,11 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E26" s="13" t="n">
-        <v>46128</v>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>46129</v>
+      <c r="E26" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="F26" s="21" t="n">
+        <v>46146</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
@@ -1748,12 +1737,12 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E27" s="7" t="n">
-        <v>46130</v>
-      </c>
-      <c r="F27" s="7" t="n">
+      <c r="E27" s="19" t="n">
         <v>46148</v>
       </c>
+      <c r="F27" s="19" t="n">
+        <v>46174</v>
+      </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
           <t>4.8</t>
@@ -1769,7 +1758,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
@@ -1794,11 +1783,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>46130</v>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>46132</v>
+      <c r="E28" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="F28" s="21" t="n">
+        <v>46153</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
@@ -1840,11 +1829,11 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E29" s="10" t="n">
-        <v>46133</v>
-      </c>
-      <c r="F29" s="10" t="n">
-        <v>46134</v>
+      <c r="E29" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>46157</v>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
@@ -1886,11 +1875,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>46135</v>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>46140</v>
+      <c r="E30" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="F30" s="21" t="n">
+        <v>46164</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
@@ -1932,11 +1921,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E31" s="10" t="n">
-        <v>46141</v>
-      </c>
-      <c r="F31" s="10" t="n">
-        <v>46142</v>
+      <c r="E31" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>46167</v>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
@@ -1978,11 +1967,11 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E32" s="13" t="n">
-        <v>46143</v>
-      </c>
-      <c r="F32" s="13" t="n">
-        <v>46144</v>
+      <c r="E32" s="21" t="n">
+        <v>46168</v>
+      </c>
+      <c r="F32" s="21" t="n">
+        <v>46169</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
@@ -2024,11 +2013,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E33" s="10" t="n">
-        <v>46145</v>
-      </c>
-      <c r="F33" s="10" t="n">
-        <v>46147</v>
+      <c r="E33" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>46172</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -2070,11 +2059,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E34" s="16" t="n">
-        <v>46148</v>
-      </c>
-      <c r="F34" s="16" t="n">
-        <v>46148</v>
+      <c r="E34" s="22" t="n">
+        <v>46174</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>46174</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2120,11 +2109,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E35" s="7" t="n">
-        <v>46149</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>46157</v>
+      <c r="E35" s="19" t="n">
+        <v>46175</v>
+      </c>
+      <c r="F35" s="19" t="n">
+        <v>46185</v>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
@@ -2141,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
@@ -2166,11 +2155,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E36" s="13" t="n">
-        <v>46149</v>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>46150</v>
+      <c r="E36" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="F36" s="21" t="n">
+        <v>46177</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
@@ -2212,11 +2201,11 @@
           <t>Alexandra Carrasco</t>
         </is>
       </c>
-      <c r="E37" s="10" t="n">
-        <v>46151</v>
-      </c>
-      <c r="F37" s="10" t="n">
-        <v>46155</v>
+      <c r="E37" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>46183</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -2258,11 +2247,11 @@
           <t>Lucas Rojas</t>
         </is>
       </c>
-      <c r="E38" s="13" t="n">
-        <v>46155</v>
-      </c>
-      <c r="F38" s="13" t="n">
-        <v>46156</v>
+      <c r="E38" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="F38" s="21" t="n">
+        <v>46185</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
@@ -2308,11 +2297,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E39" s="7" t="n">
-        <v>46157</v>
-      </c>
-      <c r="F39" s="7" t="n">
-        <v>46163</v>
+      <c r="E39" s="19" t="n">
+        <v>46186</v>
+      </c>
+      <c r="F39" s="19" t="n">
+        <v>46192</v>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
@@ -2354,15 +2343,15 @@
           <t>Allan Gálvez</t>
         </is>
       </c>
-      <c r="E40" s="13" t="n">
-        <v>46157</v>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>46161</v>
+      <c r="E40" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="F40" s="21" t="n">
+        <v>46189</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
@@ -2400,11 +2389,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E41" s="10" t="n">
-        <v>46161</v>
-      </c>
-      <c r="F41" s="10" t="n">
-        <v>46163</v>
+      <c r="E41" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>46191</v>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
@@ -2450,11 +2439,11 @@
           <t>Todos</t>
         </is>
       </c>
-      <c r="E42" s="7" t="n">
-        <v>46164</v>
-      </c>
-      <c r="F42" s="7" t="n">
-        <v>46169</v>
+      <c r="E42" s="19" t="n">
+        <v>46193</v>
+      </c>
+      <c r="F42" s="19" t="n">
+        <v>46197</v>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
@@ -2496,11 +2485,11 @@
           <t>Ricardo Silva</t>
         </is>
       </c>
-      <c r="E43" s="10" t="n">
-        <v>46164</v>
-      </c>
-      <c r="F43" s="10" t="n">
-        <v>46166</v>
+      <c r="E43" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>46195</v>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2506,7 @@
         <v>0</v>
       </c>
       <c r="K43" s="8" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
@@ -2542,11 +2531,11 @@
           <t>Alejandro Dinamarca</t>
         </is>
       </c>
-      <c r="E44" s="16" t="n">
-        <v>46169</v>
-      </c>
-      <c r="F44" s="16" t="n">
-        <v>46169</v>
+      <c r="E44" s="22" t="n">
+        <v>46197</v>
+      </c>
+      <c r="F44" s="22" t="n">
+        <v>46197</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -2587,7 +2576,7 @@
       <c r="I45" s="17" t="n"/>
       <c r="J45" s="17" t="n"/>
       <c r="K45" s="18" t="n">
-        <v>552</v>
+        <v>576</v>
       </c>
       <c r="L45" s="17" t="n"/>
     </row>

</xml_diff>